<commit_message>
T-0065: pull back 4 links the generation pilot and date audit showed were the wrong document; add pilot sheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/editorial/NTK_Backstory_Link_Review.xlsx
+++ b/editorial/NTK_Backstory_Link_Review.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G46"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2099,6 +2099,146 @@
         </is>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" s="1" t="n">
+        <v>211</v>
+      </c>
+      <c r="B47" s="1" t="inlineStr">
+        <is>
+          <t>1949</t>
+        </is>
+      </c>
+      <c r="C47" s="1" t="inlineStr">
+        <is>
+          <t>America Abroad</t>
+        </is>
+      </c>
+      <c r="D47" s="1" t="inlineStr">
+        <is>
+          <t>Speech against the North Atlantic Treaty</t>
+        </is>
+      </c>
+      <c r="E47" s="1" t="inlineStr">
+        <is>
+          <t>Robert A. Taft</t>
+        </is>
+      </c>
+      <c r="F47" s="1" t="inlineStr">
+        <is>
+          <t>Hofstadter, Great Issues in American History</t>
+        </is>
+      </c>
+      <c r="G47" s="1" t="inlineStr">
+        <is>
+          <t>PULLED 2026-10-05 after the generation pilot. Matrix date is 11 July 1949 (Taft's Senate speech against the treaty). The linked Teaching American History page is dated 26 July 1949 and opens 'Why did I vote against the Atlantic Pact?': a later speech explaining a vote already cast. Wrong document. Need the 11 July text (Congressional Record).</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="B48" s="1" t="inlineStr">
+        <is>
+          <t>1772</t>
+        </is>
+      </c>
+      <c r="C48" s="1" t="inlineStr">
+        <is>
+          <t>Power</t>
+        </is>
+      </c>
+      <c r="D48" s="1" t="inlineStr">
+        <is>
+          <t>The Advantages of the African Trade</t>
+        </is>
+      </c>
+      <c r="E48" s="1" t="inlineStr">
+        <is>
+          <t>Malachy Postlethwayt</t>
+        </is>
+      </c>
+      <c r="F48" s="1" t="inlineStr">
+        <is>
+          <t>Hofstadter, Great Issues in American History</t>
+        </is>
+      </c>
+      <c r="G48" s="1" t="inlineStr">
+        <is>
+          <t>PULLED 2026-10-05 (date audit): Matrix year 1772; the linked archive.org item is Postlethwayt's 1746 'national and private advantages of the African trade considered'. Year disagrees; may be a different work or edition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="n">
+        <v>119</v>
+      </c>
+      <c r="B49" s="1" t="inlineStr">
+        <is>
+          <t>1876</t>
+        </is>
+      </c>
+      <c r="C49" s="1" t="inlineStr">
+        <is>
+          <t>Equality</t>
+        </is>
+      </c>
+      <c r="D49" s="1" t="inlineStr">
+        <is>
+          <t>Speech in the Senate</t>
+        </is>
+      </c>
+      <c r="E49" s="1" t="inlineStr">
+        <is>
+          <t>Blanche K Bruce</t>
+        </is>
+      </c>
+      <c r="F49" s="1" t="inlineStr">
+        <is>
+          <t>Hofstadter, Great Issues in American History</t>
+        </is>
+      </c>
+      <c r="G49" s="1" t="inlineStr">
+        <is>
+          <t>PULLED 2026-10-05 (date audit): Link opens an Omeka 'has encountered an error' page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="n">
+        <v>222</v>
+      </c>
+      <c r="B50" s="1" t="inlineStr">
+        <is>
+          <t>1958</t>
+        </is>
+      </c>
+      <c r="C50" s="1" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="D50" s="1" t="inlineStr">
+        <is>
+          <t>Policy Statement of Non-Recognition of the Chinese Communist Government</t>
+        </is>
+      </c>
+      <c r="E50" s="1" t="inlineStr">
+        <is>
+          <t>State Department</t>
+        </is>
+      </c>
+      <c r="F50" s="1" t="inlineStr">
+        <is>
+          <t>Hofstadter, Great Issues in American History</t>
+        </is>
+      </c>
+      <c r="G50" s="1" t="inlineStr">
+        <is>
+          <t>PULLED 2026-10-05 (date audit): Matrix: State Dept policy statement on non-recognition of China, 10 Aug 1958. The linked page is a 1949 Foreign Relations document. Wrong period.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
T-0069: Backstory rows get 3 to 6 dated Beginnings and 3 to 5 chosen objects; object pages get About this and a View the primary document button
Selection is by rule from linked matrix objects (build_backstory.py). Text is written from the fetched source where it fits, from the matrix row alone otherwise, checked by editorial/merge_object_notes.py, all flagged unverified. Also pulls back the NATO row whose link is the treaty text, not the speech.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/editorial/NTK_Backstory_Link_Review.xlsx
+++ b/editorial/NTK_Backstory_Link_Review.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2239,6 +2239,41 @@
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>210</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>1949</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>America Abroad</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Speech for the North Atlantic Treaty</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Dean Acheson</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Hofstadter, Great Issues in American History</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>PULLED 2026-10-05 (generation pass): the matrix object is a speech; the editor-supplied Avalon page (nato.asp) is the treaty text, not a speech.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>